<commit_message>
Match source alternating section backgrounds across all pages
Split the section background variants so intro/mood/sustain use the base
paper tone and learn/feed/voices/alt use the darker paper-2, and tag the
beverages, cafe, and blog sections with the `alt` style so their bands
alternate exactly like the original site.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-beverages.report.xlsx
+++ b/tools/importer/reports/import-beverages.report.xlsx
@@ -52,7 +52,7 @@
     <t>beverages</t>
   </si>
   <si>
-    <t>2026-07-15T07:24:15.144Z</t>
+    <t>2026-07-15T09:51:39.015Z</t>
   </si>
   <si>
     <t/>
@@ -109,7 +109,7 @@
     <t>home</t>
   </si>
   <si>
-    <t>2026-07-15T07:08:51.322Z</t>
+    <t>2026-07-15T08:53:11.807Z</t>
   </si>
   <si>
     <t>Fréscopa Atelier — Every morning, perfected.</t>

</xml_diff>

<commit_message>
Refine design fidelity across dark CTA, header, footer, and category features
Add scroll-reveal animations, style the image-less dark CTA band and category
page headers, correct the brand logo and nav centering, align footer proportions,
and fix category feature blocks (image recovery + pill CTAs) to match the source.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-beverages.report.xlsx
+++ b/tools/importer/reports/import-beverages.report.xlsx
@@ -52,7 +52,7 @@
     <t>beverages</t>
   </si>
   <si>
-    <t>2026-07-15T09:51:39.015Z</t>
+    <t>2026-07-15T23:45:17.273Z</t>
   </si>
   <si>
     <t/>
@@ -73,7 +73,7 @@
     <t>blog</t>
   </si>
   <si>
-    <t>2026-07-15T07:09:05.875Z</t>
+    <t>2026-07-15T09:51:48.266Z</t>
   </si>
   <si>
     <t>https://markszulc.github.io/frescopa-atelier/blog.html</t>
@@ -91,7 +91,7 @@
     <t>cafe</t>
   </si>
   <si>
-    <t>2026-07-15T07:09:01.080Z</t>
+    <t>2026-07-15T23:26:18.079Z</t>
   </si>
   <si>
     <t>https://markszulc.github.io/frescopa-atelier/cafe.html</t>

</xml_diff>